<commit_message>
feat: implement project table pagination, restrict file upload types, and update base64 configuration handling
</commit_message>
<xml_diff>
--- a/public/template/config_sample_template.xlsx
+++ b/public/template/config_sample_template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Section</t>
   </si>
@@ -39,7 +39,7 @@
     <t>ExtractConciseOutput</t>
   </si>
   <si>
-    <t>Commercial Terms</t>
+    <t>PPA</t>
   </si>
   <si>
     <t>Contract Name</t>
@@ -57,31 +57,25 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Contract Effective Date</t>
-  </si>
-  <si>
-    <t>Contract Effective Date of the agreement</t>
-  </si>
-  <si>
-    <t>Contract Amendments
-and Dates</t>
-  </si>
-  <si>
-    <t>Contract Amendments
-and Dates  of the agreement</t>
-  </si>
-  <si>
-    <t>Contract Amendments
-and Dates of the agreement</t>
-  </si>
-  <si>
-    <t>Off-Taker</t>
-  </si>
-  <si>
-    <t>Off-Taker of the agreement</t>
+    <t xml:space="preserve">Original Effective Date </t>
+  </si>
+  <si>
+    <t>Original Effective Date  of the agreement</t>
+  </si>
+  <si>
+    <t>Amendment</t>
+  </si>
+  <si>
+    <t>Amendment  of the agreement</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Buyer</t>
+  </si>
+  <si>
+    <t>Buyer of the agreement</t>
   </si>
   <si>
     <t>Seller</t>
@@ -90,47 +84,70 @@
     <t>Seller of the agreement</t>
   </si>
   <si>
-    <t>Technical Contract Parameters</t>
-  </si>
-  <si>
-    <t>Commercial Operation
+    <t>Expected Commercial
+Operation Date</t>
+  </si>
+  <si>
+    <t>Guaranteed
+Commercial Operation
 Date</t>
   </si>
   <si>
-    <t>Schedule LDs</t>
-  </si>
-  <si>
     <t>Product</t>
   </si>
   <si>
     <t>Product info of the agreement</t>
   </si>
   <si>
-    <t>PPA Capacity</t>
-  </si>
-  <si>
-    <t>PPA Capacity info of the agreement</t>
-  </si>
-  <si>
-    <t>Purchase Price</t>
-  </si>
-  <si>
-    <t>Delivery Point</t>
-  </si>
-  <si>
-    <t>Delivery Requirements</t>
-  </si>
-  <si>
-    <t>Contracted Quantity</t>
-  </si>
-  <si>
-    <t>Availability Guarantee</t>
+    <t>Delay Damages</t>
+  </si>
+  <si>
+    <t>Delay Damages info of the agreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity Shortfall
+Damages </t>
+  </si>
+  <si>
+    <t>Capacity Shortfall
+Damages info of the agreement</t>
+  </si>
+  <si>
+    <t>Contract Price</t>
+  </si>
+  <si>
+    <t>Contract Price of the agreement</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guaranteed Availability
+Factor </t>
+  </si>
+  <si>
+    <t>Liquidated Damages</t>
+  </si>
+  <si>
+    <t>Financial Curtailment</t>
+  </si>
+  <si>
+    <t>Financial Curtailment, marginal price, Cumulative spend</t>
   </si>
   <si>
     <t>Curtailment Provisions</t>
   </si>
   <si>
-    <t>Events of Default or Termination</t>
+    <t xml:space="preserve">Development Security </t>
+  </si>
+  <si>
+    <t>Development Security</t>
+  </si>
+  <si>
+    <t>Operational Security</t>
+  </si>
+  <si>
+    <t>Operational Security, security, buyer credit support, development security</t>
   </si>
   <si>
     <t>Events of Default</t>
@@ -154,24 +171,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF91CF4F"/>
-        <bgColor rgb="FF91CF4F"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -188,27 +193,15 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -229,7 +222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="17.0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21.86"/>
@@ -272,7 +265,7 @@
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -291,24 +284,24 @@
         <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" customHeight="1" ht="17.0">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3" s="1">
         <v>10.0</v>
@@ -317,24 +310,24 @@
         <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" ht="33.0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>19</v>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="F4" s="1">
         <v>10.0</v>
@@ -343,24 +336,24 @@
         <v>13</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" ht="17.0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" ht="17.0" customFormat="1" s="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F5" s="1">
         <v>10.0</v>
@@ -369,24 +362,24 @@
         <v>13</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" customHeight="1" ht="17.0">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F6" s="1">
         <v>10.0</v>
@@ -395,50 +388,50 @@
         <v>13</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" ht="33.0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" ht="17.0">
       <c r="A7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>25</v>
+        <v>8</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>25</v>
+      <c r="E7" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="F7" s="1">
-        <v>20.0</v>
+        <v>10.0</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customHeight="1" ht="17.0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" ht="29.0">
       <c r="A8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>26</v>
+      <c r="E8" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="F8" s="1">
         <v>20.0</v>
@@ -447,24 +440,24 @@
         <v>13</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" customHeight="1" ht="17.0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" customHeight="1" ht="33.0">
       <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>28</v>
+      <c r="C9" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>27</v>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="F9" s="1">
         <v>20.0</v>
@@ -476,21 +469,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" customHeight="1" ht="17.0" customFormat="1" s="1">
+    <row r="10" customHeight="1" ht="17.0">
       <c r="A10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>29</v>
+        <v>8</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F10" s="1">
         <v>20.0</v>
@@ -502,11 +495,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" customHeight="1" ht="17.0">
+    <row r="11" customHeight="1" ht="17.0" customFormat="1" s="1">
       <c r="A11" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -528,21 +521,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" customHeight="1" ht="17.0">
+    <row r="12" customHeight="1" ht="27.0">
       <c r="A12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>31</v>
+      <c r="E12" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="F12" s="1">
         <v>20.0</v>
@@ -556,10 +549,10 @@
     </row>
     <row r="13" customHeight="1" ht="17.0">
       <c r="A13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>32</v>
+        <v>8</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>32</v>
@@ -580,21 +573,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" customHeight="1" ht="17.0">
+    <row r="14" customHeight="1" ht="17.0" customFormat="1" s="1">
       <c r="A14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F14" s="1">
         <v>30.0</v>
@@ -606,21 +599,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" customHeight="1" ht="17.0">
+    <row r="15" customHeight="1" ht="27.0" customFormat="1" s="1">
       <c r="A15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>35</v>
+        <v>8</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>35</v>
+      <c r="E15" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="F15" s="1">
         <v>30.0</v>
@@ -632,21 +625,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" customHeight="1" ht="17.0">
+    <row r="16" customHeight="1" ht="27.0" customFormat="1" s="1">
       <c r="A16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>36</v>
+        <v>8</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F16" s="1">
         <v>30.0</v>
@@ -660,22 +653,22 @@
     </row>
     <row r="17" customHeight="1" ht="17.0">
       <c r="A17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="D17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F17" s="1">
-        <v>40.0</v>
+        <v>30.0</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>13</v>
@@ -686,27 +679,131 @@
     </row>
     <row r="18" customHeight="1" ht="17.0">
       <c r="A18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="1">
+        <v>30.0</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" customHeight="1" ht="17.0">
+      <c r="A19" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F18">
+      <c r="D19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="1">
         <v>40.0</v>
       </c>
-      <c r="G18" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="1" t="s">
+      <c r="G19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" customHeight="1" ht="17.0">
+      <c r="A20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="1">
+        <v>40.0</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customHeight="1" ht="17.0">
+      <c r="A21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F21" s="1">
+        <v>50.0</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" customHeight="1" ht="17.0">
+      <c r="A22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F22" s="1">
+        <v>50.0</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>